<commit_message>
Sistemato data.json e test case 452 e 449
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#DRAGOTTAXX/DRAGOTTA GIUSEPPE/HYPER LAB/3.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#DRAGOTTAXX/DRAGOTTA GIUSEPPE/HYPER LAB/3.0/report-checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francesco\Desktop\GATEWAY\A1#111#DRAGOTTAXX\DRAGOTTA GIUSEPPE\HYPER LAB\3.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.1.100\fse\jwt\GATEWAY\A1#111#DRAGOTTAXX\DRAGOTTA GIUSEPPE\HYPER LAB\3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE22AE64-7BC8-4A36-9550-2580A8D2FF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9996C9C1-EB6E-4F95-A9A0-F74E409E3D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -858,15 +858,6 @@
     <t>2.16.840.1.113883.2.9.2.190.4.4.761d1b7e61dd10836af6185d19a8ed6b97ee2dd0fa44cb1508810a70b1ac18ed.ec006910ff^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-18T15:29:43</t>
-  </si>
-  <si>
-    <t>2e815ac72cd2507261d52c12b8aaf6cc</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.190.4.4.be40251f12d8d4ded097d457fef2c13eee3077e2a9bc7dc6e1e4dbf5248ecb2c.20bf5f693f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-18T15:36:34</t>
   </si>
   <si>
@@ -894,15 +885,6 @@
     <t>2.16.840.1.113883.2.9.2.190.4.4.8f8994b2b490283c0cbab45e9a61af51520386549d6476cad1ffdd23e3153c99.b188c24d1c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-18T15:43:28</t>
-  </si>
-  <si>
-    <t>e9e2039f70cc337ad3a319a4d93007f5</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.190.4.4.8f8994b2b490283c0cbab45e9a61af51520386549d6476cad1ffdd23e3153c99.b72cc2f589^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-18T15:47:51</t>
   </si>
   <si>
@@ -919,6 +901,24 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.190.4.4.8f8994b2b490283c0cbab45e9a61af51520386549d6476cad1ffdd23e3153c99.b72aa259a3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-21T13:31:02</t>
+  </si>
+  <si>
+    <t>6948b61380dc5065d59dd4e0fc02b23a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.190.4.4.be40251f12d8d4ded097d457fef2c13eee3077e2a9bc7dc6e1e4dbf5248ecb2c.d266fdec03^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-21T13:41:07</t>
+  </si>
+  <si>
+    <t>f6f692d5c2366da48e79f4bdcd88f999</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.190.4.4.8f8994b2b490283c0cbab45e9a61af51520386549d6476cad1ffdd23e3153c99.c2ec691de3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -1494,28 +1494,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1525,12 +1503,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1625,6 +1597,34 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
@@ -1951,7 +1951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="300" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="285" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -3102,14 +3102,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="37" t="s">
+      <c r="B2" s="77"/>
+      <c r="C2" s="72" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="50"/>
+      <c r="D2" s="73"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -3130,14 +3130,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="44" t="s">
+      <c r="B3" s="79"/>
+      <c r="C3" s="70" t="s">
         <v>183</v>
       </c>
-      <c r="D3" s="49"/>
+      <c r="D3" s="71"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -3158,12 +3158,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="44" t="s">
+      <c r="A4" s="80"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="70" t="s">
         <v>184</v>
       </c>
-      <c r="D4" s="49"/>
+      <c r="D4" s="71"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -3185,12 +3185,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42"/>
-      <c r="B5" s="43"/>
-      <c r="C5" s="44" t="s">
+      <c r="A5" s="82"/>
+      <c r="B5" s="83"/>
+      <c r="C5" s="70" t="s">
         <v>185</v>
       </c>
-      <c r="D5" s="49"/>
+      <c r="D5" s="71"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -3211,8 +3211,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="34"/>
+      <c r="A6" s="74"/>
+      <c r="B6" s="75"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -3347,1779 +3347,1779 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="51">
+    <row r="10" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="37">
         <v>4</v>
       </c>
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="52" t="s">
+      <c r="C10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="53" t="s">
+      <c r="D10" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="54" t="s">
+      <c r="E10" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="81">
+      <c r="F10" s="67">
         <v>46099</v>
       </c>
-      <c r="G10" s="53" t="s">
+      <c r="G10" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="H10" s="53" t="s">
+      <c r="H10" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="I10" s="53" t="s">
+      <c r="I10" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="J10" s="56" t="s">
+      <c r="J10" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56" t="s">
+      <c r="K10" s="42"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="N10" s="56"/>
-      <c r="O10" s="56"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="56"/>
-      <c r="R10" s="56"/>
-      <c r="S10" s="56"/>
-      <c r="T10" s="56"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="58"/>
-      <c r="W10" s="56" t="s">
+      <c r="N10" s="42"/>
+      <c r="O10" s="42"/>
+      <c r="P10" s="42"/>
+      <c r="Q10" s="42"/>
+      <c r="R10" s="42"/>
+      <c r="S10" s="42"/>
+      <c r="T10" s="42"/>
+      <c r="U10" s="43"/>
+      <c r="V10" s="44"/>
+      <c r="W10" s="42" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="53">
+    <row r="11" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="39">
         <v>28</v>
       </c>
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="53" t="s">
+      <c r="D11" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="54" t="s">
+      <c r="E11" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="61"/>
-      <c r="J11" s="56" t="s">
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="47"/>
+      <c r="J11" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K11" s="56" t="s">
+      <c r="K11" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
-      <c r="N11" s="56"/>
-      <c r="O11" s="56"/>
-      <c r="P11" s="56"/>
-      <c r="Q11" s="56"/>
-      <c r="R11" s="56"/>
-      <c r="S11" s="56"/>
-      <c r="T11" s="56"/>
-      <c r="U11" s="57"/>
-      <c r="V11" s="58"/>
-      <c r="W11" s="56" t="s">
+      <c r="L11" s="42"/>
+      <c r="M11" s="42"/>
+      <c r="N11" s="42"/>
+      <c r="O11" s="42"/>
+      <c r="P11" s="42"/>
+      <c r="Q11" s="42"/>
+      <c r="R11" s="42"/>
+      <c r="S11" s="42"/>
+      <c r="T11" s="42"/>
+      <c r="U11" s="43"/>
+      <c r="V11" s="44"/>
+      <c r="W11" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="53">
+    <row r="12" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="39">
         <v>36</v>
       </c>
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="60" t="s">
+      <c r="C12" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="53" t="s">
+      <c r="D12" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="54" t="s">
+      <c r="E12" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="56" t="s">
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="47"/>
+      <c r="J12" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K12" s="56" t="s">
+      <c r="K12" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
-      <c r="N12" s="56"/>
-      <c r="O12" s="56"/>
-      <c r="P12" s="56"/>
-      <c r="Q12" s="56"/>
-      <c r="R12" s="56"/>
-      <c r="S12" s="56"/>
-      <c r="T12" s="56"/>
-      <c r="U12" s="57"/>
-      <c r="V12" s="58"/>
-      <c r="W12" s="56" t="s">
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="42"/>
+      <c r="P12" s="42"/>
+      <c r="Q12" s="42"/>
+      <c r="R12" s="42"/>
+      <c r="S12" s="42"/>
+      <c r="T12" s="42"/>
+      <c r="U12" s="43"/>
+      <c r="V12" s="44"/>
+      <c r="W12" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="53">
+    <row r="13" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="39">
         <v>44</v>
       </c>
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="60" t="s">
+      <c r="C13" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="53" t="s">
+      <c r="D13" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="54" t="s">
+      <c r="E13" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="55">
+      <c r="F13" s="41">
         <v>46099</v>
       </c>
-      <c r="G13" s="55" t="s">
+      <c r="G13" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="H13" s="55"/>
-      <c r="I13" s="61"/>
-      <c r="J13" s="56" t="s">
+      <c r="H13" s="41"/>
+      <c r="I13" s="47"/>
+      <c r="J13" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="K13" s="56"/>
-      <c r="L13" s="56"/>
-      <c r="M13" s="56" t="s">
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="N13" s="56" t="s">
+      <c r="N13" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="O13" s="56"/>
-      <c r="P13" s="56" t="s">
+      <c r="O13" s="42"/>
+      <c r="P13" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="Q13" s="56" t="s">
+      <c r="Q13" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="R13" s="56"/>
-      <c r="S13" s="56" t="s">
+      <c r="R13" s="42"/>
+      <c r="S13" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="T13" s="56"/>
-      <c r="U13" s="57"/>
-      <c r="V13" s="58"/>
-      <c r="W13" s="56" t="s">
+      <c r="T13" s="42"/>
+      <c r="U13" s="43"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="53">
+    <row r="14" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="39">
         <v>53</v>
       </c>
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="60" t="s">
+      <c r="C14" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="53" t="s">
+      <c r="D14" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="54" t="s">
+      <c r="E14" s="40" t="s">
         <v>67</v>
       </c>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="61"/>
-      <c r="J14" s="56" t="s">
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K14" s="56" t="s">
+      <c r="K14" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="56"/>
-      <c r="O14" s="56"/>
-      <c r="P14" s="56"/>
-      <c r="Q14" s="56"/>
-      <c r="R14" s="56"/>
-      <c r="S14" s="56"/>
-      <c r="T14" s="56"/>
-      <c r="U14" s="57"/>
-      <c r="V14" s="58"/>
-      <c r="W14" s="56" t="s">
+      <c r="L14" s="42"/>
+      <c r="M14" s="42"/>
+      <c r="N14" s="42"/>
+      <c r="O14" s="42"/>
+      <c r="P14" s="42"/>
+      <c r="Q14" s="42"/>
+      <c r="R14" s="42"/>
+      <c r="S14" s="42"/>
+      <c r="T14" s="42"/>
+      <c r="U14" s="43"/>
+      <c r="V14" s="44"/>
+      <c r="W14" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="53">
+    <row r="15" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="39">
         <v>55</v>
       </c>
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="60" t="s">
+      <c r="C15" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="53" t="s">
+      <c r="D15" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="54" t="s">
+      <c r="E15" s="40" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="61"/>
-      <c r="J15" s="56" t="s">
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K15" s="56" t="s">
+      <c r="K15" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L15" s="56"/>
-      <c r="M15" s="56"/>
-      <c r="N15" s="56"/>
-      <c r="O15" s="56"/>
-      <c r="P15" s="56"/>
-      <c r="Q15" s="56"/>
-      <c r="R15" s="56"/>
-      <c r="S15" s="56"/>
-      <c r="T15" s="56"/>
-      <c r="U15" s="57"/>
-      <c r="V15" s="58"/>
-      <c r="W15" s="56" t="s">
+      <c r="L15" s="42"/>
+      <c r="M15" s="42"/>
+      <c r="N15" s="42"/>
+      <c r="O15" s="42"/>
+      <c r="P15" s="42"/>
+      <c r="Q15" s="42"/>
+      <c r="R15" s="42"/>
+      <c r="S15" s="42"/>
+      <c r="T15" s="42"/>
+      <c r="U15" s="43"/>
+      <c r="V15" s="44"/>
+      <c r="W15" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="53">
+    <row r="16" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="39">
         <v>56</v>
       </c>
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="60" t="s">
+      <c r="C16" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="53" t="s">
+      <c r="D16" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="E16" s="54" t="s">
+      <c r="E16" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="56" t="s">
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K16" s="56" t="s">
+      <c r="K16" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="56"/>
-      <c r="O16" s="56"/>
-      <c r="P16" s="56"/>
-      <c r="Q16" s="56"/>
-      <c r="R16" s="56"/>
-      <c r="S16" s="56"/>
-      <c r="T16" s="56"/>
-      <c r="U16" s="57"/>
-      <c r="V16" s="58"/>
-      <c r="W16" s="56" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="42"/>
+      <c r="N16" s="42"/>
+      <c r="O16" s="42"/>
+      <c r="P16" s="42"/>
+      <c r="Q16" s="42"/>
+      <c r="R16" s="42"/>
+      <c r="S16" s="42"/>
+      <c r="T16" s="42"/>
+      <c r="U16" s="43"/>
+      <c r="V16" s="44"/>
+      <c r="W16" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="53">
+    <row r="17" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="39">
         <v>57</v>
       </c>
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="60" t="s">
+      <c r="C17" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="53" t="s">
+      <c r="D17" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="54" t="s">
+      <c r="E17" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="56" t="s">
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K17" s="56" t="s">
+      <c r="K17" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="56"/>
-      <c r="O17" s="56"/>
-      <c r="P17" s="56"/>
-      <c r="Q17" s="56"/>
-      <c r="R17" s="56"/>
-      <c r="S17" s="56"/>
-      <c r="T17" s="56"/>
-      <c r="U17" s="57"/>
-      <c r="V17" s="58"/>
-      <c r="W17" s="56" t="s">
+      <c r="L17" s="42"/>
+      <c r="M17" s="42"/>
+      <c r="N17" s="42"/>
+      <c r="O17" s="42"/>
+      <c r="P17" s="42"/>
+      <c r="Q17" s="42"/>
+      <c r="R17" s="42"/>
+      <c r="S17" s="42"/>
+      <c r="T17" s="42"/>
+      <c r="U17" s="43"/>
+      <c r="V17" s="44"/>
+      <c r="W17" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="53">
+    <row r="18" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="39">
         <v>59</v>
       </c>
-      <c r="B18" s="53" t="s">
+      <c r="B18" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="53" t="s">
+      <c r="D18" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="E18" s="54" t="s">
+      <c r="E18" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="56" t="s">
+      <c r="F18" s="41"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="47"/>
+      <c r="J18" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K18" s="56" t="s">
+      <c r="K18" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L18" s="56"/>
-      <c r="M18" s="56"/>
-      <c r="N18" s="56"/>
-      <c r="O18" s="56"/>
-      <c r="P18" s="56"/>
-      <c r="Q18" s="56"/>
-      <c r="R18" s="56"/>
-      <c r="S18" s="56"/>
-      <c r="T18" s="56"/>
-      <c r="U18" s="57"/>
-      <c r="V18" s="58"/>
-      <c r="W18" s="56" t="s">
+      <c r="L18" s="42"/>
+      <c r="M18" s="42"/>
+      <c r="N18" s="42"/>
+      <c r="O18" s="42"/>
+      <c r="P18" s="42"/>
+      <c r="Q18" s="42"/>
+      <c r="R18" s="42"/>
+      <c r="S18" s="42"/>
+      <c r="T18" s="42"/>
+      <c r="U18" s="43"/>
+      <c r="V18" s="44"/>
+      <c r="W18" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="53">
+    <row r="19" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="39">
         <v>60</v>
       </c>
-      <c r="B19" s="53" t="s">
+      <c r="B19" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="60" t="s">
+      <c r="C19" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="53" t="s">
+      <c r="D19" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="54" t="s">
+      <c r="E19" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="55">
+      <c r="F19" s="41">
         <v>46099</v>
       </c>
-      <c r="G19" s="55" t="s">
+      <c r="G19" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="H19" s="41" t="s">
+        <v>195</v>
+      </c>
+      <c r="I19" s="47" t="s">
+        <v>196</v>
+      </c>
+      <c r="J19" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="K19" s="42"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="N19" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="O19" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="P19" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q19" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="R19" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="S19" s="42" t="s">
+        <v>188</v>
+      </c>
+      <c r="T19" s="42"/>
+      <c r="U19" s="43"/>
+      <c r="V19" s="44"/>
+      <c r="W19" s="42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="39">
+        <v>61</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="K20" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
+      <c r="R20" s="42"/>
+      <c r="S20" s="42"/>
+      <c r="T20" s="42"/>
+      <c r="U20" s="43"/>
+      <c r="V20" s="44"/>
+      <c r="W20" s="42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="39">
+        <v>62</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="47"/>
+      <c r="J21" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="K21" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="L21" s="42"/>
+      <c r="M21" s="42"/>
+      <c r="N21" s="42"/>
+      <c r="O21" s="42"/>
+      <c r="P21" s="42"/>
+      <c r="Q21" s="42"/>
+      <c r="R21" s="42"/>
+      <c r="S21" s="42"/>
+      <c r="T21" s="42"/>
+      <c r="U21" s="43"/>
+      <c r="V21" s="44"/>
+      <c r="W21" s="42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" s="65" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="57">
+        <v>191</v>
+      </c>
+      <c r="B22" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="57" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="59" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="60"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="62" t="s">
+        <v>181</v>
+      </c>
+      <c r="K22" s="62" t="s">
+        <v>138</v>
+      </c>
+      <c r="L22" s="62"/>
+      <c r="M22" s="62"/>
+      <c r="N22" s="62"/>
+      <c r="O22" s="62"/>
+      <c r="P22" s="62"/>
+      <c r="Q22" s="62"/>
+      <c r="R22" s="62"/>
+      <c r="S22" s="62"/>
+      <c r="T22" s="62"/>
+      <c r="U22" s="63"/>
+      <c r="V22" s="64"/>
+      <c r="W22" s="62" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" s="65" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="57">
+        <v>376</v>
+      </c>
+      <c r="B23" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="57" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="59" t="s">
+        <v>115</v>
+      </c>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="62" t="s">
+        <v>181</v>
+      </c>
+      <c r="K23" s="62" t="s">
+        <v>138</v>
+      </c>
+      <c r="L23" s="62"/>
+      <c r="M23" s="62"/>
+      <c r="N23" s="62"/>
+      <c r="O23" s="62"/>
+      <c r="P23" s="62"/>
+      <c r="Q23" s="62"/>
+      <c r="R23" s="62"/>
+      <c r="S23" s="62"/>
+      <c r="T23" s="62"/>
+      <c r="U23" s="63"/>
+      <c r="V23" s="64"/>
+      <c r="W23" s="62" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="39">
+        <v>452</v>
+      </c>
+      <c r="B24" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="F24" s="67">
+        <v>46102</v>
+      </c>
+      <c r="G24" s="39" t="s">
+        <v>209</v>
+      </c>
+      <c r="H24" s="68" t="s">
+        <v>210</v>
+      </c>
+      <c r="I24" s="39" t="s">
+        <v>211</v>
+      </c>
+      <c r="J24" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="K24" s="42"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="N24" s="42"/>
+      <c r="O24" s="42"/>
+      <c r="P24" s="42"/>
+      <c r="Q24" s="42"/>
+      <c r="R24" s="42"/>
+      <c r="S24" s="42"/>
+      <c r="T24" s="42"/>
+      <c r="U24" s="43"/>
+      <c r="V24" s="44"/>
+      <c r="W24" s="42" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="39">
+        <v>466</v>
+      </c>
+      <c r="B25" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="E25" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="K25" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="L25" s="39"/>
+      <c r="M25" s="42"/>
+      <c r="N25" s="42"/>
+      <c r="O25" s="39"/>
+      <c r="P25" s="42"/>
+      <c r="Q25" s="42"/>
+      <c r="R25" s="42"/>
+      <c r="S25" s="39"/>
+      <c r="T25" s="42"/>
+      <c r="U25" s="39"/>
+      <c r="V25" s="39"/>
+      <c r="W25" s="39" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" s="45" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="39">
+        <v>473</v>
+      </c>
+      <c r="B26" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="E26" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="F26" s="41">
+        <v>46099</v>
+      </c>
+      <c r="G26" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="H19" s="55" t="s">
+      <c r="H26" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="I19" s="61" t="s">
+      <c r="I26" s="47" t="s">
         <v>199</v>
       </c>
-      <c r="J19" s="56" t="s">
+      <c r="J26" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
-      <c r="M19" s="56" t="s">
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="N19" s="56" t="s">
+      <c r="N26" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="O19" s="56" t="s">
+      <c r="O26" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="P19" s="56" t="s">
+      <c r="P26" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="Q19" s="56" t="s">
+      <c r="Q26" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="R19" s="56" t="s">
+      <c r="R26" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="S19" s="56" t="s">
+      <c r="S26" s="42" t="s">
         <v>188</v>
       </c>
-      <c r="T19" s="56"/>
-      <c r="U19" s="57"/>
-      <c r="V19" s="58"/>
-      <c r="W19" s="56" t="s">
+      <c r="T26" s="42"/>
+      <c r="U26" s="43"/>
+      <c r="V26" s="44"/>
+      <c r="W26" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="53">
+    <row r="27" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="48">
+        <v>32</v>
+      </c>
+      <c r="B27" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K27" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L27" s="53"/>
+      <c r="M27" s="53"/>
+      <c r="N27" s="53"/>
+      <c r="O27" s="53"/>
+      <c r="P27" s="53"/>
+      <c r="Q27" s="53"/>
+      <c r="R27" s="53"/>
+      <c r="S27" s="53"/>
+      <c r="T27" s="53"/>
+      <c r="U27" s="54"/>
+      <c r="V27" s="55"/>
+      <c r="W27" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="48">
+        <v>40</v>
+      </c>
+      <c r="B28" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="53" t="s">
+      <c r="E28" s="50" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" s="51"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="52"/>
+      <c r="J28" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K28" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L28" s="53"/>
+      <c r="M28" s="53"/>
+      <c r="N28" s="53"/>
+      <c r="O28" s="53"/>
+      <c r="P28" s="53"/>
+      <c r="Q28" s="53"/>
+      <c r="R28" s="53"/>
+      <c r="S28" s="53"/>
+      <c r="T28" s="53"/>
+      <c r="U28" s="54"/>
+      <c r="V28" s="55"/>
+      <c r="W28" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="48">
+        <v>48</v>
+      </c>
+      <c r="B29" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="54" t="s">
-        <v>79</v>
-      </c>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="61"/>
-      <c r="J20" s="56" t="s">
+      <c r="C29" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D29" s="48" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="51">
+        <v>46099</v>
+      </c>
+      <c r="G29" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="H29" s="66"/>
+      <c r="I29" s="52"/>
+      <c r="J29" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="K29" s="53"/>
+      <c r="L29" s="53"/>
+      <c r="M29" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="K20" s="56" t="s">
+      <c r="N29" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="O29" s="53"/>
+      <c r="P29" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q29" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="R29" s="53"/>
+      <c r="S29" s="53" t="s">
+        <v>186</v>
+      </c>
+      <c r="T29" s="53"/>
+      <c r="U29" s="54"/>
+      <c r="V29" s="55"/>
+      <c r="W29" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="48">
+        <v>152</v>
+      </c>
+      <c r="B30" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D30" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>83</v>
+      </c>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="51"/>
+      <c r="I30" s="52"/>
+      <c r="J30" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K30" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="L20" s="56"/>
-      <c r="M20" s="56"/>
-      <c r="N20" s="56"/>
-      <c r="O20" s="56"/>
-      <c r="P20" s="56"/>
-      <c r="Q20" s="56"/>
-      <c r="R20" s="56"/>
-      <c r="S20" s="56"/>
-      <c r="T20" s="56"/>
-      <c r="U20" s="57"/>
-      <c r="V20" s="58"/>
-      <c r="W20" s="56" t="s">
+      <c r="L30" s="53"/>
+      <c r="M30" s="53"/>
+      <c r="N30" s="53"/>
+      <c r="O30" s="53"/>
+      <c r="P30" s="53"/>
+      <c r="Q30" s="53"/>
+      <c r="R30" s="53"/>
+      <c r="S30" s="53"/>
+      <c r="T30" s="53"/>
+      <c r="U30" s="54"/>
+      <c r="V30" s="55"/>
+      <c r="W30" s="53" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="53">
-        <v>62</v>
-      </c>
-      <c r="B21" s="53" t="s">
+    <row r="31" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="48">
+        <v>154</v>
+      </c>
+      <c r="B31" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="53" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="61"/>
-      <c r="J21" s="56" t="s">
+      <c r="C31" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="48" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="F31" s="51"/>
+      <c r="G31" s="51"/>
+      <c r="H31" s="51"/>
+      <c r="I31" s="52"/>
+      <c r="J31" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="K21" s="56" t="s">
+      <c r="K31" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="L21" s="56"/>
-      <c r="M21" s="56"/>
-      <c r="N21" s="56"/>
-      <c r="O21" s="56"/>
-      <c r="P21" s="56"/>
-      <c r="Q21" s="56"/>
-      <c r="R21" s="56"/>
-      <c r="S21" s="56"/>
-      <c r="T21" s="56"/>
-      <c r="U21" s="57"/>
-      <c r="V21" s="58"/>
-      <c r="W21" s="56" t="s">
+      <c r="L31" s="53"/>
+      <c r="M31" s="53"/>
+      <c r="N31" s="53"/>
+      <c r="O31" s="53"/>
+      <c r="P31" s="53"/>
+      <c r="Q31" s="53"/>
+      <c r="R31" s="53"/>
+      <c r="S31" s="53"/>
+      <c r="T31" s="53"/>
+      <c r="U31" s="54"/>
+      <c r="V31" s="55"/>
+      <c r="W31" s="53" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:23" s="79" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="71">
-        <v>191</v>
-      </c>
-      <c r="B22" s="71" t="s">
+    <row r="32" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="48">
+        <v>155</v>
+      </c>
+      <c r="B32" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="72" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="71" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" s="73" t="s">
-        <v>113</v>
-      </c>
-      <c r="F22" s="74"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="74"/>
-      <c r="I22" s="75"/>
-      <c r="J22" s="76" t="s">
+      <c r="C32" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D32" s="48" t="s">
+        <v>86</v>
+      </c>
+      <c r="E32" s="50" t="s">
+        <v>87</v>
+      </c>
+      <c r="F32" s="51"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="52"/>
+      <c r="J32" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="K22" s="76" t="s">
-        <v>138</v>
-      </c>
-      <c r="L22" s="76"/>
-      <c r="M22" s="76"/>
-      <c r="N22" s="76"/>
-      <c r="O22" s="76"/>
-      <c r="P22" s="76"/>
-      <c r="Q22" s="76"/>
-      <c r="R22" s="76"/>
-      <c r="S22" s="76"/>
-      <c r="T22" s="76"/>
-      <c r="U22" s="77"/>
-      <c r="V22" s="78"/>
-      <c r="W22" s="76" t="s">
+      <c r="K32" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L32" s="53"/>
+      <c r="M32" s="53"/>
+      <c r="N32" s="53"/>
+      <c r="O32" s="53"/>
+      <c r="P32" s="53"/>
+      <c r="Q32" s="53"/>
+      <c r="R32" s="53"/>
+      <c r="S32" s="53"/>
+      <c r="T32" s="53"/>
+      <c r="U32" s="54"/>
+      <c r="V32" s="55"/>
+      <c r="W32" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="48">
+        <v>156</v>
+      </c>
+      <c r="B33" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="F33" s="51"/>
+      <c r="G33" s="51"/>
+      <c r="H33" s="51"/>
+      <c r="I33" s="52"/>
+      <c r="J33" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K33" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L33" s="53"/>
+      <c r="M33" s="53"/>
+      <c r="N33" s="53"/>
+      <c r="O33" s="53"/>
+      <c r="P33" s="53"/>
+      <c r="Q33" s="53"/>
+      <c r="R33" s="53"/>
+      <c r="S33" s="53"/>
+      <c r="T33" s="53"/>
+      <c r="U33" s="54"/>
+      <c r="V33" s="55"/>
+      <c r="W33" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="48">
+        <v>159</v>
+      </c>
+      <c r="B34" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D34" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="50" t="s">
+        <v>91</v>
+      </c>
+      <c r="F34" s="51"/>
+      <c r="G34" s="51"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="52"/>
+      <c r="J34" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K34" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L34" s="53"/>
+      <c r="M34" s="53"/>
+      <c r="N34" s="53"/>
+      <c r="O34" s="53"/>
+      <c r="P34" s="53"/>
+      <c r="Q34" s="53"/>
+      <c r="R34" s="53"/>
+      <c r="S34" s="53"/>
+      <c r="T34" s="53"/>
+      <c r="U34" s="54"/>
+      <c r="V34" s="55"/>
+      <c r="W34" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="48">
+        <v>160</v>
+      </c>
+      <c r="B35" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D35" s="48" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="F35" s="51"/>
+      <c r="G35" s="51"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="52"/>
+      <c r="J35" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K35" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L35" s="53"/>
+      <c r="M35" s="53"/>
+      <c r="N35" s="53"/>
+      <c r="O35" s="53"/>
+      <c r="P35" s="53"/>
+      <c r="Q35" s="53"/>
+      <c r="R35" s="53"/>
+      <c r="S35" s="53"/>
+      <c r="T35" s="53"/>
+      <c r="U35" s="54"/>
+      <c r="V35" s="55"/>
+      <c r="W35" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="48">
+        <v>161</v>
+      </c>
+      <c r="B36" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D36" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36" s="51"/>
+      <c r="G36" s="51"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="52"/>
+      <c r="J36" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K36" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L36" s="53"/>
+      <c r="M36" s="53"/>
+      <c r="N36" s="53"/>
+      <c r="O36" s="53"/>
+      <c r="P36" s="53"/>
+      <c r="Q36" s="53"/>
+      <c r="R36" s="53"/>
+      <c r="S36" s="53"/>
+      <c r="T36" s="53"/>
+      <c r="U36" s="54"/>
+      <c r="V36" s="55"/>
+      <c r="W36" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="48">
+        <v>162</v>
+      </c>
+      <c r="B37" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="E37" s="50" t="s">
+        <v>97</v>
+      </c>
+      <c r="F37" s="51"/>
+      <c r="G37" s="51"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="52"/>
+      <c r="J37" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K37" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L37" s="53"/>
+      <c r="M37" s="53"/>
+      <c r="N37" s="53"/>
+      <c r="O37" s="53"/>
+      <c r="P37" s="53"/>
+      <c r="Q37" s="53"/>
+      <c r="R37" s="53"/>
+      <c r="S37" s="53"/>
+      <c r="T37" s="53"/>
+      <c r="U37" s="54"/>
+      <c r="V37" s="55"/>
+      <c r="W37" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="48">
+        <v>163</v>
+      </c>
+      <c r="B38" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D38" s="48" t="s">
+        <v>98</v>
+      </c>
+      <c r="E38" s="50" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="51"/>
+      <c r="G38" s="51"/>
+      <c r="H38" s="51"/>
+      <c r="I38" s="52"/>
+      <c r="J38" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K38" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L38" s="53"/>
+      <c r="M38" s="53"/>
+      <c r="N38" s="53"/>
+      <c r="O38" s="53"/>
+      <c r="P38" s="53"/>
+      <c r="Q38" s="53"/>
+      <c r="R38" s="53"/>
+      <c r="S38" s="53"/>
+      <c r="T38" s="53"/>
+      <c r="U38" s="54"/>
+      <c r="V38" s="55"/>
+      <c r="W38" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="48">
+        <v>164</v>
+      </c>
+      <c r="B39" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="48" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="F39" s="51"/>
+      <c r="G39" s="51"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="52"/>
+      <c r="J39" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K39" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L39" s="53"/>
+      <c r="M39" s="53"/>
+      <c r="N39" s="53"/>
+      <c r="O39" s="53"/>
+      <c r="P39" s="53"/>
+      <c r="Q39" s="53"/>
+      <c r="R39" s="53"/>
+      <c r="S39" s="53"/>
+      <c r="T39" s="53"/>
+      <c r="U39" s="54"/>
+      <c r="V39" s="55"/>
+      <c r="W39" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="48">
+        <v>165</v>
+      </c>
+      <c r="B40" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="F40" s="51"/>
+      <c r="G40" s="51"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="52"/>
+      <c r="J40" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K40" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L40" s="53"/>
+      <c r="M40" s="53"/>
+      <c r="N40" s="53"/>
+      <c r="O40" s="53"/>
+      <c r="P40" s="53"/>
+      <c r="Q40" s="53"/>
+      <c r="R40" s="53"/>
+      <c r="S40" s="53"/>
+      <c r="T40" s="53"/>
+      <c r="U40" s="54"/>
+      <c r="V40" s="55"/>
+      <c r="W40" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="48">
+        <v>166</v>
+      </c>
+      <c r="B41" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D41" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="E41" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" s="51"/>
+      <c r="G41" s="51"/>
+      <c r="H41" s="51"/>
+      <c r="I41" s="52"/>
+      <c r="J41" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K41" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L41" s="53"/>
+      <c r="M41" s="53"/>
+      <c r="N41" s="53"/>
+      <c r="O41" s="53"/>
+      <c r="P41" s="53"/>
+      <c r="Q41" s="53"/>
+      <c r="R41" s="53"/>
+      <c r="S41" s="53"/>
+      <c r="T41" s="53"/>
+      <c r="U41" s="54"/>
+      <c r="V41" s="55"/>
+      <c r="W41" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="48">
+        <v>167</v>
+      </c>
+      <c r="B42" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D42" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="E42" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="F42" s="51"/>
+      <c r="G42" s="51"/>
+      <c r="H42" s="51"/>
+      <c r="I42" s="52"/>
+      <c r="J42" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K42" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L42" s="53"/>
+      <c r="M42" s="53"/>
+      <c r="N42" s="53"/>
+      <c r="O42" s="53"/>
+      <c r="P42" s="53"/>
+      <c r="Q42" s="53"/>
+      <c r="R42" s="53"/>
+      <c r="S42" s="53"/>
+      <c r="T42" s="53"/>
+      <c r="U42" s="54"/>
+      <c r="V42" s="55"/>
+      <c r="W42" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="48">
+        <v>168</v>
+      </c>
+      <c r="B43" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C43" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="E43" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F43" s="51">
+        <v>46099</v>
+      </c>
+      <c r="G43" s="51" t="s">
+        <v>206</v>
+      </c>
+      <c r="H43" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="I43" s="52" t="s">
+        <v>208</v>
+      </c>
+      <c r="J43" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="K43" s="53"/>
+      <c r="L43" s="53"/>
+      <c r="M43" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="N43" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="O43" s="53" t="s">
+        <v>187</v>
+      </c>
+      <c r="P43" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q43" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="R43" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="S43" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="T43" s="53"/>
+      <c r="U43" s="54"/>
+      <c r="V43" s="55"/>
+      <c r="W43" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="48">
+        <v>169</v>
+      </c>
+      <c r="B44" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D44" s="48" t="s">
+        <v>110</v>
+      </c>
+      <c r="E44" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="F44" s="51"/>
+      <c r="G44" s="51"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="52"/>
+      <c r="J44" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="K44" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="L44" s="53"/>
+      <c r="M44" s="53"/>
+      <c r="N44" s="53"/>
+      <c r="O44" s="53"/>
+      <c r="P44" s="53"/>
+      <c r="Q44" s="53"/>
+      <c r="R44" s="53"/>
+      <c r="S44" s="53"/>
+      <c r="T44" s="53"/>
+      <c r="U44" s="54"/>
+      <c r="V44" s="55"/>
+      <c r="W44" s="53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="48">
+        <v>448</v>
+      </c>
+      <c r="B45" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D45" s="48" t="s">
+        <v>117</v>
+      </c>
+      <c r="E45" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="F45" s="69">
+        <v>46099</v>
+      </c>
+      <c r="G45" s="48" t="s">
+        <v>200</v>
+      </c>
+      <c r="H45" s="48" t="s">
+        <v>201</v>
+      </c>
+      <c r="I45" s="48" t="s">
+        <v>202</v>
+      </c>
+      <c r="J45" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="K45" s="53"/>
+      <c r="L45" s="53"/>
+      <c r="M45" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="N45" s="53"/>
+      <c r="O45" s="53"/>
+      <c r="P45" s="53"/>
+      <c r="Q45" s="53"/>
+      <c r="R45" s="53"/>
+      <c r="S45" s="53"/>
+      <c r="T45" s="53"/>
+      <c r="U45" s="54"/>
+      <c r="V45" s="55"/>
+      <c r="W45" s="53" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:23" s="79" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="71">
-        <v>376</v>
-      </c>
-      <c r="B23" s="71" t="s">
+    <row r="46" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="48">
+        <v>449</v>
+      </c>
+      <c r="B46" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="72" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="E23" s="73" t="s">
-        <v>115</v>
-      </c>
-      <c r="F23" s="74"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="74"/>
-      <c r="I23" s="75"/>
-      <c r="J23" s="76" t="s">
+      <c r="C46" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46" s="48" t="s">
+        <v>119</v>
+      </c>
+      <c r="E46" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="69">
+        <v>46102</v>
+      </c>
+      <c r="G46" s="48" t="s">
+        <v>212</v>
+      </c>
+      <c r="H46" s="48" t="s">
+        <v>213</v>
+      </c>
+      <c r="I46" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="J46" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="K46" s="53"/>
+      <c r="L46" s="53"/>
+      <c r="M46" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="K23" s="76" t="s">
-        <v>138</v>
-      </c>
-      <c r="L23" s="76"/>
-      <c r="M23" s="76"/>
-      <c r="N23" s="76"/>
-      <c r="O23" s="76"/>
-      <c r="P23" s="76"/>
-      <c r="Q23" s="76"/>
-      <c r="R23" s="76"/>
-      <c r="S23" s="76"/>
-      <c r="T23" s="76"/>
-      <c r="U23" s="77"/>
-      <c r="V23" s="78"/>
-      <c r="W23" s="76" t="s">
+      <c r="N46" s="53"/>
+      <c r="O46" s="53"/>
+      <c r="P46" s="53"/>
+      <c r="Q46" s="53"/>
+      <c r="R46" s="53"/>
+      <c r="S46" s="53"/>
+      <c r="T46" s="53"/>
+      <c r="U46" s="54"/>
+      <c r="V46" s="55"/>
+      <c r="W46" s="53" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="53">
-        <v>452</v>
-      </c>
-      <c r="B24" s="53" t="s">
+    <row r="47" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="48">
+        <v>461</v>
+      </c>
+      <c r="B47" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="E24" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="F24" s="81">
+      <c r="C47" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D47" s="48" t="s">
+        <v>123</v>
+      </c>
+      <c r="E47" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="F47" s="69">
         <v>46099</v>
       </c>
-      <c r="G24" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="H24" s="82" t="s">
-        <v>195</v>
-      </c>
-      <c r="I24" s="53" t="s">
-        <v>196</v>
-      </c>
-      <c r="J24" s="56" t="s">
+      <c r="G47" s="48" t="s">
+        <v>203</v>
+      </c>
+      <c r="H47" s="48" t="s">
+        <v>204</v>
+      </c>
+      <c r="I47" s="48" t="s">
+        <v>205</v>
+      </c>
+      <c r="J47" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="K24" s="56"/>
-      <c r="L24" s="56"/>
-      <c r="M24" s="56" t="s">
+      <c r="K47" s="53"/>
+      <c r="L47" s="48"/>
+      <c r="M47" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="N47" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="O47" s="48" t="s">
+        <v>187</v>
+      </c>
+      <c r="P47" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="N24" s="56"/>
-      <c r="O24" s="56"/>
-      <c r="P24" s="56"/>
-      <c r="Q24" s="56"/>
-      <c r="R24" s="56"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="56"/>
-      <c r="U24" s="57"/>
-      <c r="V24" s="58"/>
-      <c r="W24" s="56" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="53">
-        <v>466</v>
-      </c>
-      <c r="B25" s="53" t="s">
+      <c r="Q47" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="R47" s="53" t="s">
+        <v>181</v>
+      </c>
+      <c r="S47" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="T47" s="53"/>
+      <c r="U47" s="48"/>
+      <c r="V47" s="48"/>
+      <c r="W47" s="48" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="48">
+        <v>468</v>
+      </c>
+      <c r="B48" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="53" t="s">
-        <v>125</v>
-      </c>
-      <c r="E25" s="54" t="s">
-        <v>126</v>
-      </c>
-      <c r="F25" s="53"/>
-      <c r="G25" s="53"/>
-      <c r="H25" s="53"/>
-      <c r="I25" s="60"/>
-      <c r="J25" s="56" t="s">
+      <c r="C48" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D48" s="49" t="s">
+        <v>127</v>
+      </c>
+      <c r="E48" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+      <c r="H48" s="48"/>
+      <c r="I48" s="49"/>
+      <c r="J48" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="K25" s="56" t="s">
+      <c r="K48" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="L25" s="53"/>
-      <c r="M25" s="56"/>
-      <c r="N25" s="56"/>
-      <c r="O25" s="53"/>
-      <c r="P25" s="56"/>
-      <c r="Q25" s="56"/>
-      <c r="R25" s="56"/>
-      <c r="S25" s="53"/>
-      <c r="T25" s="56"/>
-      <c r="U25" s="53"/>
-      <c r="V25" s="53"/>
-      <c r="W25" s="53" t="s">
+      <c r="L48" s="48"/>
+      <c r="M48" s="53"/>
+      <c r="N48" s="53"/>
+      <c r="O48" s="48"/>
+      <c r="P48" s="53"/>
+      <c r="Q48" s="53"/>
+      <c r="R48" s="53"/>
+      <c r="S48" s="48"/>
+      <c r="T48" s="53"/>
+      <c r="U48" s="48"/>
+      <c r="V48" s="48"/>
+      <c r="W48" s="48" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:23" s="59" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="53">
-        <v>473</v>
-      </c>
-      <c r="B26" s="53" t="s">
+    <row r="49" spans="1:23" s="56" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="48">
+        <v>475</v>
+      </c>
+      <c r="B49" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D26" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="E26" s="54" t="s">
-        <v>130</v>
-      </c>
-      <c r="F26" s="55">
-        <v>46099</v>
-      </c>
-      <c r="G26" s="55" t="s">
-        <v>200</v>
-      </c>
-      <c r="H26" s="55" t="s">
-        <v>201</v>
-      </c>
-      <c r="I26" s="61" t="s">
-        <v>202</v>
-      </c>
-      <c r="J26" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="K26" s="56"/>
-      <c r="L26" s="56"/>
-      <c r="M26" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="N26" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="O26" s="56" t="s">
-        <v>187</v>
-      </c>
-      <c r="P26" s="56" t="s">
+      <c r="C49" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D49" s="48" t="s">
+        <v>131</v>
+      </c>
+      <c r="E49" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="52"/>
+      <c r="J49" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="Q26" s="56" t="s">
-        <v>181</v>
-      </c>
-      <c r="R26" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="S26" s="56" t="s">
-        <v>188</v>
-      </c>
-      <c r="T26" s="56"/>
-      <c r="U26" s="57"/>
-      <c r="V26" s="58"/>
-      <c r="W26" s="56" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="62">
-        <v>32</v>
-      </c>
-      <c r="B27" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="E27" s="64" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" s="65"/>
-      <c r="G27" s="65"/>
-      <c r="H27" s="65"/>
-      <c r="I27" s="66"/>
-      <c r="J27" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K27" s="67" t="s">
+      <c r="K49" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="L27" s="67"/>
-      <c r="M27" s="67"/>
-      <c r="N27" s="67"/>
-      <c r="O27" s="67"/>
-      <c r="P27" s="67"/>
-      <c r="Q27" s="67"/>
-      <c r="R27" s="67"/>
-      <c r="S27" s="67"/>
-      <c r="T27" s="67"/>
-      <c r="U27" s="68"/>
-      <c r="V27" s="69"/>
-      <c r="W27" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="62">
-        <v>40</v>
-      </c>
-      <c r="B28" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D28" s="62" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="64" t="s">
-        <v>60</v>
-      </c>
-      <c r="F28" s="65"/>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K28" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L28" s="67"/>
-      <c r="M28" s="67"/>
-      <c r="N28" s="67"/>
-      <c r="O28" s="67"/>
-      <c r="P28" s="67"/>
-      <c r="Q28" s="67"/>
-      <c r="R28" s="67"/>
-      <c r="S28" s="67"/>
-      <c r="T28" s="67"/>
-      <c r="U28" s="68"/>
-      <c r="V28" s="69"/>
-      <c r="W28" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="62">
-        <v>48</v>
-      </c>
-      <c r="B29" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D29" s="62" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="64" t="s">
-        <v>63</v>
-      </c>
-      <c r="F29" s="65">
-        <v>46099</v>
-      </c>
-      <c r="G29" s="65" t="s">
-        <v>190</v>
-      </c>
-      <c r="H29" s="80"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K29" s="67"/>
-      <c r="L29" s="67"/>
-      <c r="M29" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="N29" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="O29" s="67"/>
-      <c r="P29" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q29" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="R29" s="67"/>
-      <c r="S29" s="67" t="s">
-        <v>186</v>
-      </c>
-      <c r="T29" s="67"/>
-      <c r="U29" s="68"/>
-      <c r="V29" s="69"/>
-      <c r="W29" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="62">
-        <v>152</v>
-      </c>
-      <c r="B30" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D30" s="62" t="s">
-        <v>82</v>
-      </c>
-      <c r="E30" s="64" t="s">
-        <v>83</v>
-      </c>
-      <c r="F30" s="65"/>
-      <c r="G30" s="65"/>
-      <c r="H30" s="65"/>
-      <c r="I30" s="66"/>
-      <c r="J30" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K30" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L30" s="67"/>
-      <c r="M30" s="67"/>
-      <c r="N30" s="67"/>
-      <c r="O30" s="67"/>
-      <c r="P30" s="67"/>
-      <c r="Q30" s="67"/>
-      <c r="R30" s="67"/>
-      <c r="S30" s="67"/>
-      <c r="T30" s="67"/>
-      <c r="U30" s="68"/>
-      <c r="V30" s="69"/>
-      <c r="W30" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="62">
-        <v>154</v>
-      </c>
-      <c r="B31" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D31" s="62" t="s">
-        <v>84</v>
-      </c>
-      <c r="E31" s="64" t="s">
-        <v>85</v>
-      </c>
-      <c r="F31" s="65"/>
-      <c r="G31" s="65"/>
-      <c r="H31" s="65"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K31" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L31" s="67"/>
-      <c r="M31" s="67"/>
-      <c r="N31" s="67"/>
-      <c r="O31" s="67"/>
-      <c r="P31" s="67"/>
-      <c r="Q31" s="67"/>
-      <c r="R31" s="67"/>
-      <c r="S31" s="67"/>
-      <c r="T31" s="67"/>
-      <c r="U31" s="68"/>
-      <c r="V31" s="69"/>
-      <c r="W31" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="62">
-        <v>155</v>
-      </c>
-      <c r="B32" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D32" s="62" t="s">
-        <v>86</v>
-      </c>
-      <c r="E32" s="64" t="s">
-        <v>87</v>
-      </c>
-      <c r="F32" s="65"/>
-      <c r="G32" s="65"/>
-      <c r="H32" s="65"/>
-      <c r="I32" s="66"/>
-      <c r="J32" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K32" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L32" s="67"/>
-      <c r="M32" s="67"/>
-      <c r="N32" s="67"/>
-      <c r="O32" s="67"/>
-      <c r="P32" s="67"/>
-      <c r="Q32" s="67"/>
-      <c r="R32" s="67"/>
-      <c r="S32" s="67"/>
-      <c r="T32" s="67"/>
-      <c r="U32" s="68"/>
-      <c r="V32" s="69"/>
-      <c r="W32" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="62">
-        <v>156</v>
-      </c>
-      <c r="B33" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D33" s="62" t="s">
-        <v>88</v>
-      </c>
-      <c r="E33" s="64" t="s">
-        <v>89</v>
-      </c>
-      <c r="F33" s="65"/>
-      <c r="G33" s="65"/>
-      <c r="H33" s="65"/>
-      <c r="I33" s="66"/>
-      <c r="J33" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K33" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L33" s="67"/>
-      <c r="M33" s="67"/>
-      <c r="N33" s="67"/>
-      <c r="O33" s="67"/>
-      <c r="P33" s="67"/>
-      <c r="Q33" s="67"/>
-      <c r="R33" s="67"/>
-      <c r="S33" s="67"/>
-      <c r="T33" s="67"/>
-      <c r="U33" s="68"/>
-      <c r="V33" s="69"/>
-      <c r="W33" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="62">
-        <v>159</v>
-      </c>
-      <c r="B34" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D34" s="62" t="s">
-        <v>90</v>
-      </c>
-      <c r="E34" s="64" t="s">
-        <v>91</v>
-      </c>
-      <c r="F34" s="65"/>
-      <c r="G34" s="65"/>
-      <c r="H34" s="65"/>
-      <c r="I34" s="66"/>
-      <c r="J34" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K34" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L34" s="67"/>
-      <c r="M34" s="67"/>
-      <c r="N34" s="67"/>
-      <c r="O34" s="67"/>
-      <c r="P34" s="67"/>
-      <c r="Q34" s="67"/>
-      <c r="R34" s="67"/>
-      <c r="S34" s="67"/>
-      <c r="T34" s="67"/>
-      <c r="U34" s="68"/>
-      <c r="V34" s="69"/>
-      <c r="W34" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="62">
-        <v>160</v>
-      </c>
-      <c r="B35" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C35" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D35" s="62" t="s">
-        <v>92</v>
-      </c>
-      <c r="E35" s="64" t="s">
-        <v>93</v>
-      </c>
-      <c r="F35" s="65"/>
-      <c r="G35" s="65"/>
-      <c r="H35" s="65"/>
-      <c r="I35" s="66"/>
-      <c r="J35" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K35" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L35" s="67"/>
-      <c r="M35" s="67"/>
-      <c r="N35" s="67"/>
-      <c r="O35" s="67"/>
-      <c r="P35" s="67"/>
-      <c r="Q35" s="67"/>
-      <c r="R35" s="67"/>
-      <c r="S35" s="67"/>
-      <c r="T35" s="67"/>
-      <c r="U35" s="68"/>
-      <c r="V35" s="69"/>
-      <c r="W35" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="62">
-        <v>161</v>
-      </c>
-      <c r="B36" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C36" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D36" s="62" t="s">
-        <v>94</v>
-      </c>
-      <c r="E36" s="64" t="s">
-        <v>95</v>
-      </c>
-      <c r="F36" s="65"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
-      <c r="I36" s="66"/>
-      <c r="J36" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K36" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L36" s="67"/>
-      <c r="M36" s="67"/>
-      <c r="N36" s="67"/>
-      <c r="O36" s="67"/>
-      <c r="P36" s="67"/>
-      <c r="Q36" s="67"/>
-      <c r="R36" s="67"/>
-      <c r="S36" s="67"/>
-      <c r="T36" s="67"/>
-      <c r="U36" s="68"/>
-      <c r="V36" s="69"/>
-      <c r="W36" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="62">
-        <v>162</v>
-      </c>
-      <c r="B37" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D37" s="62" t="s">
-        <v>96</v>
-      </c>
-      <c r="E37" s="64" t="s">
-        <v>97</v>
-      </c>
-      <c r="F37" s="65"/>
-      <c r="G37" s="65"/>
-      <c r="H37" s="65"/>
-      <c r="I37" s="66"/>
-      <c r="J37" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K37" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L37" s="67"/>
-      <c r="M37" s="67"/>
-      <c r="N37" s="67"/>
-      <c r="O37" s="67"/>
-      <c r="P37" s="67"/>
-      <c r="Q37" s="67"/>
-      <c r="R37" s="67"/>
-      <c r="S37" s="67"/>
-      <c r="T37" s="67"/>
-      <c r="U37" s="68"/>
-      <c r="V37" s="69"/>
-      <c r="W37" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="62">
-        <v>163</v>
-      </c>
-      <c r="B38" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C38" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D38" s="62" t="s">
-        <v>98</v>
-      </c>
-      <c r="E38" s="64" t="s">
-        <v>99</v>
-      </c>
-      <c r="F38" s="65"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="65"/>
-      <c r="I38" s="66"/>
-      <c r="J38" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K38" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L38" s="67"/>
-      <c r="M38" s="67"/>
-      <c r="N38" s="67"/>
-      <c r="O38" s="67"/>
-      <c r="P38" s="67"/>
-      <c r="Q38" s="67"/>
-      <c r="R38" s="67"/>
-      <c r="S38" s="67"/>
-      <c r="T38" s="67"/>
-      <c r="U38" s="68"/>
-      <c r="V38" s="69"/>
-      <c r="W38" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="62">
-        <v>164</v>
-      </c>
-      <c r="B39" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D39" s="62" t="s">
-        <v>100</v>
-      </c>
-      <c r="E39" s="64" t="s">
-        <v>101</v>
-      </c>
-      <c r="F39" s="65"/>
-      <c r="G39" s="65"/>
-      <c r="H39" s="65"/>
-      <c r="I39" s="66"/>
-      <c r="J39" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K39" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L39" s="67"/>
-      <c r="M39" s="67"/>
-      <c r="N39" s="67"/>
-      <c r="O39" s="67"/>
-      <c r="P39" s="67"/>
-      <c r="Q39" s="67"/>
-      <c r="R39" s="67"/>
-      <c r="S39" s="67"/>
-      <c r="T39" s="67"/>
-      <c r="U39" s="68"/>
-      <c r="V39" s="69"/>
-      <c r="W39" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="62">
-        <v>165</v>
-      </c>
-      <c r="B40" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C40" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40" s="62" t="s">
-        <v>102</v>
-      </c>
-      <c r="E40" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="F40" s="65"/>
-      <c r="G40" s="65"/>
-      <c r="H40" s="65"/>
-      <c r="I40" s="66"/>
-      <c r="J40" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K40" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L40" s="67"/>
-      <c r="M40" s="67"/>
-      <c r="N40" s="67"/>
-      <c r="O40" s="67"/>
-      <c r="P40" s="67"/>
-      <c r="Q40" s="67"/>
-      <c r="R40" s="67"/>
-      <c r="S40" s="67"/>
-      <c r="T40" s="67"/>
-      <c r="U40" s="68"/>
-      <c r="V40" s="69"/>
-      <c r="W40" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="41" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="62">
-        <v>166</v>
-      </c>
-      <c r="B41" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C41" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D41" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="E41" s="64" t="s">
-        <v>105</v>
-      </c>
-      <c r="F41" s="65"/>
-      <c r="G41" s="65"/>
-      <c r="H41" s="65"/>
-      <c r="I41" s="66"/>
-      <c r="J41" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K41" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L41" s="67"/>
-      <c r="M41" s="67"/>
-      <c r="N41" s="67"/>
-      <c r="O41" s="67"/>
-      <c r="P41" s="67"/>
-      <c r="Q41" s="67"/>
-      <c r="R41" s="67"/>
-      <c r="S41" s="67"/>
-      <c r="T41" s="67"/>
-      <c r="U41" s="68"/>
-      <c r="V41" s="69"/>
-      <c r="W41" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="62">
-        <v>167</v>
-      </c>
-      <c r="B42" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C42" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" s="62" t="s">
-        <v>106</v>
-      </c>
-      <c r="E42" s="64" t="s">
-        <v>107</v>
-      </c>
-      <c r="F42" s="65"/>
-      <c r="G42" s="65"/>
-      <c r="H42" s="65"/>
-      <c r="I42" s="66"/>
-      <c r="J42" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K42" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L42" s="67"/>
-      <c r="M42" s="67"/>
-      <c r="N42" s="67"/>
-      <c r="O42" s="67"/>
-      <c r="P42" s="67"/>
-      <c r="Q42" s="67"/>
-      <c r="R42" s="67"/>
-      <c r="S42" s="67"/>
-      <c r="T42" s="67"/>
-      <c r="U42" s="68"/>
-      <c r="V42" s="69"/>
-      <c r="W42" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="43" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="62">
-        <v>168</v>
-      </c>
-      <c r="B43" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C43" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D43" s="62" t="s">
-        <v>108</v>
-      </c>
-      <c r="E43" s="64" t="s">
-        <v>109</v>
-      </c>
-      <c r="F43" s="65">
-        <v>46099</v>
-      </c>
-      <c r="G43" s="65" t="s">
-        <v>212</v>
-      </c>
-      <c r="H43" s="65" t="s">
-        <v>213</v>
-      </c>
-      <c r="I43" s="66" t="s">
-        <v>214</v>
-      </c>
-      <c r="J43" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K43" s="67"/>
-      <c r="L43" s="67"/>
-      <c r="M43" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="N43" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="O43" s="67" t="s">
-        <v>187</v>
-      </c>
-      <c r="P43" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q43" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="R43" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="S43" s="67" t="s">
-        <v>188</v>
-      </c>
-      <c r="T43" s="67"/>
-      <c r="U43" s="68"/>
-      <c r="V43" s="69"/>
-      <c r="W43" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="44" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="62">
-        <v>169</v>
-      </c>
-      <c r="B44" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" s="62" t="s">
-        <v>110</v>
-      </c>
-      <c r="E44" s="64" t="s">
-        <v>111</v>
-      </c>
-      <c r="F44" s="65"/>
-      <c r="G44" s="65"/>
-      <c r="H44" s="65"/>
-      <c r="I44" s="66"/>
-      <c r="J44" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K44" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L44" s="67"/>
-      <c r="M44" s="67"/>
-      <c r="N44" s="67"/>
-      <c r="O44" s="67"/>
-      <c r="P44" s="67"/>
-      <c r="Q44" s="67"/>
-      <c r="R44" s="67"/>
-      <c r="S44" s="67"/>
-      <c r="T44" s="67"/>
-      <c r="U44" s="68"/>
-      <c r="V44" s="69"/>
-      <c r="W44" s="67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="45" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="62">
-        <v>448</v>
-      </c>
-      <c r="B45" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C45" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" s="62" t="s">
-        <v>117</v>
-      </c>
-      <c r="E45" s="64" t="s">
-        <v>118</v>
-      </c>
-      <c r="F45" s="83">
-        <v>46099</v>
-      </c>
-      <c r="G45" s="62" t="s">
-        <v>203</v>
-      </c>
-      <c r="H45" s="62" t="s">
-        <v>204</v>
-      </c>
-      <c r="I45" s="62" t="s">
-        <v>205</v>
-      </c>
-      <c r="J45" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K45" s="67"/>
-      <c r="L45" s="67"/>
-      <c r="M45" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="N45" s="67"/>
-      <c r="O45" s="67"/>
-      <c r="P45" s="67"/>
-      <c r="Q45" s="67"/>
-      <c r="R45" s="67"/>
-      <c r="S45" s="67"/>
-      <c r="T45" s="67"/>
-      <c r="U45" s="68"/>
-      <c r="V45" s="69"/>
-      <c r="W45" s="67" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="46" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="62">
-        <v>449</v>
-      </c>
-      <c r="B46" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D46" s="62" t="s">
-        <v>119</v>
-      </c>
-      <c r="E46" s="64" t="s">
-        <v>120</v>
-      </c>
-      <c r="F46" s="83">
-        <v>46099</v>
-      </c>
-      <c r="G46" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="H46" s="62" t="s">
-        <v>207</v>
-      </c>
-      <c r="I46" s="62" t="s">
-        <v>208</v>
-      </c>
-      <c r="J46" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K46" s="67"/>
-      <c r="L46" s="67"/>
-      <c r="M46" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="N46" s="67"/>
-      <c r="O46" s="67"/>
-      <c r="P46" s="67"/>
-      <c r="Q46" s="67"/>
-      <c r="R46" s="67"/>
-      <c r="S46" s="67"/>
-      <c r="T46" s="67"/>
-      <c r="U46" s="68"/>
-      <c r="V46" s="69"/>
-      <c r="W46" s="67" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="47" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="62">
-        <v>461</v>
-      </c>
-      <c r="B47" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C47" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D47" s="62" t="s">
-        <v>123</v>
-      </c>
-      <c r="E47" s="64" t="s">
-        <v>124</v>
-      </c>
-      <c r="F47" s="83">
-        <v>46099</v>
-      </c>
-      <c r="G47" s="62" t="s">
-        <v>209</v>
-      </c>
-      <c r="H47" s="62" t="s">
-        <v>210</v>
-      </c>
-      <c r="I47" s="62" t="s">
-        <v>211</v>
-      </c>
-      <c r="J47" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K47" s="67"/>
-      <c r="L47" s="62"/>
-      <c r="M47" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="N47" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="O47" s="62" t="s">
-        <v>187</v>
-      </c>
-      <c r="P47" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q47" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="R47" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="S47" s="67" t="s">
-        <v>188</v>
-      </c>
-      <c r="T47" s="67"/>
-      <c r="U47" s="62"/>
-      <c r="V47" s="62"/>
-      <c r="W47" s="62" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="62">
-        <v>468</v>
-      </c>
-      <c r="B48" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D48" s="63" t="s">
-        <v>127</v>
-      </c>
-      <c r="E48" s="64" t="s">
-        <v>128</v>
-      </c>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="63"/>
-      <c r="J48" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K48" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L48" s="62"/>
-      <c r="M48" s="67"/>
-      <c r="N48" s="67"/>
-      <c r="O48" s="62"/>
-      <c r="P48" s="67"/>
-      <c r="Q48" s="67"/>
-      <c r="R48" s="67"/>
-      <c r="S48" s="62"/>
-      <c r="T48" s="67"/>
-      <c r="U48" s="62"/>
-      <c r="V48" s="62"/>
-      <c r="W48" s="62" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="49" spans="1:23" s="70" customFormat="1" ht="150" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="62">
-        <v>475</v>
-      </c>
-      <c r="B49" s="62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C49" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D49" s="62" t="s">
-        <v>131</v>
-      </c>
-      <c r="E49" s="64" t="s">
-        <v>132</v>
-      </c>
-      <c r="F49" s="65"/>
-      <c r="G49" s="65"/>
-      <c r="H49" s="65"/>
-      <c r="I49" s="66"/>
-      <c r="J49" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K49" s="67" t="s">
-        <v>143</v>
-      </c>
-      <c r="L49" s="67"/>
-      <c r="M49" s="67"/>
-      <c r="N49" s="67"/>
-      <c r="O49" s="67"/>
-      <c r="P49" s="67"/>
-      <c r="Q49" s="67"/>
-      <c r="R49" s="67"/>
-      <c r="S49" s="67"/>
-      <c r="T49" s="67"/>
-      <c r="U49" s="68"/>
-      <c r="V49" s="69"/>
-      <c r="W49" s="67" t="s">
+      <c r="L49" s="53"/>
+      <c r="M49" s="53"/>
+      <c r="N49" s="53"/>
+      <c r="O49" s="53"/>
+      <c r="P49" s="53"/>
+      <c r="Q49" s="53"/>
+      <c r="R49" s="53"/>
+      <c r="S49" s="53"/>
+      <c r="T49" s="53"/>
+      <c r="U49" s="54"/>
+      <c r="V49" s="55"/>
+      <c r="W49" s="53" t="s">
         <v>50</v>
       </c>
     </row>
@@ -8229,16 +8229,16 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="36" t="s">
         <v>152</v>
       </c>
     </row>
@@ -8313,16 +8313,16 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="45" t="s">
+      <c r="A8" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="D8" s="47" t="s">
+      <c r="D8" s="35" t="s">
         <v>164</v>
       </c>
     </row>
@@ -10421,6 +10421,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -10684,42 +10705,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10742,9 +10731,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>